<commit_message>
Split Maf_Maf_Hay_140 and Maf_Nor_Man_40 on Distribution_Zone14_9_2026
Cut the two zones along YWC zone boundaries on the 14/9/2026 layer,
name parts with the recheck-list codes (_A/_B), and add the full layer
with the split applied and Zone_Code set for the 10 listed zones.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JAu1NnEtyFdpjqezLDmDLJ
</commit_message>
<xml_diff>
--- a/Recheck/Zones_Recheck_List_Answered.xlsx
+++ b/Recheck/Zones_Recheck_List_Answered.xlsx
@@ -1816,7 +1816,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
@@ -2321,7 +2320,7 @@
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>Cut along YWC zones 96/97 (66% / 34%). Operator confirmed mixed supply. CHECK: 42% of Hay Aggad is above 716 m while the Balaama tank is at ~736 m - gravity pressure weak there; sources may be swapped between A and B. Confirm with operator.</t>
+          <t>Cut along YWC zones 96/97 (63% / 37% on Distribution_Zone14_9_2026). Operator confirmed mixed supply. CHECK: 42% of Hay Aggad is above 716 m while the Balaama tank is at ~736 m - gravity pressure weak there; sources may be swapped between A and B. Confirm with operator.</t>
         </is>
       </c>
       <c r="N13" t="n">
@@ -2399,7 +2398,7 @@
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t>Cut along YWC zones 26/30 (68% / 32%). The Sabha part is in YWC zone 30 (SABHA, Sabha PS), which also covers GIS zone 108 Sabha (P_Zone Sabha_PS).</t>
+          <t>Cut along YWC zones 26/30 (59% / 41% on Distribution_Zone14_9_2026). The Sabha part is in YWC zone 30 (SABHA, Sabha PS), which also covers GIS zone 108 Sabha (P_Zone Sabha_PS).</t>
         </is>
       </c>
       <c r="N15" t="n">

</xml_diff>